<commit_message>
refactorización completa de los bots
</commit_message>
<xml_diff>
--- a/Oficios.xlsx
+++ b/Oficios.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="30">
   <si>
     <t xml:space="preserve">Folio Sugo</t>
   </si>
@@ -35,9 +35,6 @@
   </si>
   <si>
     <t xml:space="preserve">Dictamen Wizard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Informe</t>
   </si>
   <si>
     <t xml:space="preserve">Fecha Cierre</t>
@@ -215,7 +212,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -469,13 +466,14 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="19.79"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="26.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -497,134 +495,131 @@
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="24.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="B2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>9</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>12</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="E4" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="24.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="B5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="C5" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>23</v>
-      </c>
       <c r="C7" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="C8" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>26</v>
-      </c>
       <c r="E8" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>28</v>
-      </c>
       <c r="C9" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>30</v>
-      </c>
       <c r="C10" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>